<commit_message>
update snap + food insecurity w 2025 data
</commit_message>
<xml_diff>
--- a/visuals/info_table.xlsx
+++ b/visuals/info_table.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="209">
   <si>
     <t xml:space="preserve">Community District</t>
   </si>
@@ -32,7 +32,7 @@
     <t xml:space="preserve">100,929</t>
   </si>
   <si>
-    <t xml:space="preserve">46,452</t>
+    <t xml:space="preserve">46,014</t>
   </si>
   <si>
     <t xml:space="preserve">46%</t>
@@ -44,10 +44,10 @@
     <t xml:space="preserve"> 54,454</t>
   </si>
   <si>
-    <t xml:space="preserve">23,596</t>
-  </si>
-  <si>
-    <t xml:space="preserve">43%</t>
+    <t xml:space="preserve">22,794</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42%</t>
   </si>
   <si>
     <t xml:space="preserve">B03</t>
@@ -56,10 +56,10 @@
     <t xml:space="preserve"> 93,755</t>
   </si>
   <si>
-    <t xml:space="preserve">44,591</t>
-  </si>
-  <si>
-    <t xml:space="preserve">48%</t>
+    <t xml:space="preserve">43,642</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47%</t>
   </si>
   <si>
     <t xml:space="preserve">B04</t>
@@ -68,10 +68,10 @@
     <t xml:space="preserve">150,436</t>
   </si>
   <si>
-    <t xml:space="preserve">59,454</t>
-  </si>
-  <si>
-    <t xml:space="preserve">40%</t>
+    <t xml:space="preserve">58,144</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39%</t>
   </si>
   <si>
     <t xml:space="preserve">B05</t>
@@ -80,7 +80,7 @@
     <t xml:space="preserve">132,584</t>
   </si>
   <si>
-    <t xml:space="preserve">57,057</t>
+    <t xml:space="preserve">55,868</t>
   </si>
   <si>
     <t xml:space="preserve">B06</t>
@@ -89,7 +89,10 @@
     <t xml:space="preserve"> 89,216</t>
   </si>
   <si>
-    <t xml:space="preserve">40,871</t>
+    <t xml:space="preserve">39,878</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45%</t>
   </si>
   <si>
     <t xml:space="preserve">B07</t>
@@ -98,10 +101,10 @@
     <t xml:space="preserve">146,813</t>
   </si>
   <si>
-    <t xml:space="preserve">50,675</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35%</t>
+    <t xml:space="preserve">50,067</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34%</t>
   </si>
   <si>
     <t xml:space="preserve">B08</t>
@@ -110,7 +113,7 @@
     <t xml:space="preserve">106,924</t>
   </si>
   <si>
-    <t xml:space="preserve">19,718</t>
+    <t xml:space="preserve">19,702</t>
   </si>
   <si>
     <t xml:space="preserve">18%</t>
@@ -122,7 +125,7 @@
     <t xml:space="preserve">188,249</t>
   </si>
   <si>
-    <t xml:space="preserve">59,121</t>
+    <t xml:space="preserve">57,656</t>
   </si>
   <si>
     <t xml:space="preserve">31%</t>
@@ -134,7 +137,7 @@
     <t xml:space="preserve">130,763</t>
   </si>
   <si>
-    <t xml:space="preserve">22,331</t>
+    <t xml:space="preserve">22,567</t>
   </si>
   <si>
     <t xml:space="preserve">17%</t>
@@ -146,7 +149,7 @@
     <t xml:space="preserve">119,666</t>
   </si>
   <si>
-    <t xml:space="preserve">28,535</t>
+    <t xml:space="preserve">28,792</t>
   </si>
   <si>
     <t xml:space="preserve">24%</t>
@@ -158,7 +161,7 @@
     <t xml:space="preserve">163,489</t>
   </si>
   <si>
-    <t xml:space="preserve">44,432</t>
+    <t xml:space="preserve">44,754</t>
   </si>
   <si>
     <t xml:space="preserve">27%</t>
@@ -170,7 +173,7 @@
     <t xml:space="preserve">204,125</t>
   </si>
   <si>
-    <t xml:space="preserve">52,989</t>
+    <t xml:space="preserve">53,694</t>
   </si>
   <si>
     <t xml:space="preserve">26%</t>
@@ -182,7 +185,7 @@
     <t xml:space="preserve">130,021</t>
   </si>
   <si>
-    <t xml:space="preserve">14,539</t>
+    <t xml:space="preserve">14,330</t>
   </si>
   <si>
     <t xml:space="preserve">11%</t>
@@ -194,7 +197,7 @@
     <t xml:space="preserve">174,960</t>
   </si>
   <si>
-    <t xml:space="preserve">45,544</t>
+    <t xml:space="preserve">45,496</t>
   </si>
   <si>
     <t xml:space="preserve">K04</t>
@@ -203,336 +206,333 @@
     <t xml:space="preserve">120,747</t>
   </si>
   <si>
-    <t xml:space="preserve">23,611</t>
+    <t xml:space="preserve">22,447</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200,293</t>
+  </si>
+  <si>
+    <t xml:space="preserve">66,887</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">113,933</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10,011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">133,230</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23,112</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">108,259</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20,201</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">102,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22,223</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">136,071</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20,058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">198,870</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42,019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">205,377</t>
+  </si>
+  <si>
+    <t xml:space="preserve">72,954</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">108,905</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34,151</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">164,568</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34,969</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">169,632</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33,309</t>
   </si>
   <si>
     <t xml:space="preserve">20%</t>
   </si>
   <si>
-    <t xml:space="preserve">K05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">200,293</t>
-  </si>
-  <si>
-    <t xml:space="preserve">67,860</t>
-  </si>
-  <si>
-    <t xml:space="preserve">34%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">113,933</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10,347</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">133,230</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24,082</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">108,259</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20,221</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">102,000</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22,573</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">136,071</t>
+    <t xml:space="preserve">K16</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 98,506</t>
+  </si>
+  <si>
+    <t xml:space="preserve">37,297</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">162,446</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35,480</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">204,095</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32,478</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M01</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 78,390</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2,193</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M02</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 92,445</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2,893</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">163,141</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36,631</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">131,351</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14,004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M05</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 63,600</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 5,531</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">155,614</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 7,464</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">222,129</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17,042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">231,983</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 6,913</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">110,458</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22,012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">130,440</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30,823</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">125,771</t>
+  </si>
+  <si>
+    <t xml:space="preserve">41,971</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">180,206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47,829</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">196,803</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26,630</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">137,981</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13,205</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">179,134</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25,425</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">181,025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28,606</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">178,178</t>
   </si>
   <si>
     <t xml:space="preserve">20,634</t>
   </si>
   <si>
-    <t xml:space="preserve">15%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">198,870</t>
-  </si>
-  <si>
-    <t xml:space="preserve">43,667</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">205,377</t>
-  </si>
-  <si>
-    <t xml:space="preserve">70,678</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">108,905</t>
-  </si>
-  <si>
-    <t xml:space="preserve">34,910</t>
-  </si>
-  <si>
-    <t xml:space="preserve">32%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">164,568</t>
-  </si>
-  <si>
-    <t xml:space="preserve">36,181</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">169,632</t>
-  </si>
-  <si>
-    <t xml:space="preserve">33,797</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K16</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 98,506</t>
-  </si>
-  <si>
-    <t xml:space="preserve">37,764</t>
-  </si>
-  <si>
-    <t xml:space="preserve">38%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">162,446</t>
-  </si>
-  <si>
-    <t xml:space="preserve">36,368</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">204,095</t>
-  </si>
-  <si>
-    <t xml:space="preserve">33,540</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M01</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 78,390</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 2,163</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M02</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 92,445</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 3,055</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">163,141</t>
-  </si>
-  <si>
-    <t xml:space="preserve">37,735</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">131,351</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14,118</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M05</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 63,600</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 5,736</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">155,614</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 6,794</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">222,129</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17,464</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">231,983</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 6,750</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">110,458</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22,937</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">130,440</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31,435</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">125,771</t>
-  </si>
-  <si>
-    <t xml:space="preserve">43,304</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">180,206</t>
-  </si>
-  <si>
-    <t xml:space="preserve">49,241</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">196,803</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27,141</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">137,981</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13,122</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">179,134</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26,968</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">181,025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29,837</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">178,178</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21,785</t>
-  </si>
-  <si>
     <t xml:space="preserve">12%</t>
   </si>
   <si>
@@ -542,7 +542,7 @@
     <t xml:space="preserve">120,955</t>
   </si>
   <si>
-    <t xml:space="preserve">13,872</t>
+    <t xml:space="preserve">14,111</t>
   </si>
   <si>
     <t xml:space="preserve">Q07</t>
@@ -551,7 +551,7 @@
     <t xml:space="preserve">269,587</t>
   </si>
   <si>
-    <t xml:space="preserve">38,498</t>
+    <t xml:space="preserve">38,431</t>
   </si>
   <si>
     <t xml:space="preserve">Q08</t>
@@ -560,7 +560,7 @@
     <t xml:space="preserve">161,402</t>
   </si>
   <si>
-    <t xml:space="preserve">23,193</t>
+    <t xml:space="preserve">23,079</t>
   </si>
   <si>
     <t xml:space="preserve">Q09</t>
@@ -569,7 +569,7 @@
     <t xml:space="preserve">152,839</t>
   </si>
   <si>
-    <t xml:space="preserve">26,803</t>
+    <t xml:space="preserve">26,116</t>
   </si>
   <si>
     <t xml:space="preserve">Q10</t>
@@ -578,7 +578,7 @@
     <t xml:space="preserve">129,411</t>
   </si>
   <si>
-    <t xml:space="preserve">19,510</t>
+    <t xml:space="preserve">19,401</t>
   </si>
   <si>
     <t xml:space="preserve">Q11</t>
@@ -587,7 +587,7 @@
     <t xml:space="preserve">122,211</t>
   </si>
   <si>
-    <t xml:space="preserve">10,428</t>
+    <t xml:space="preserve">10,421</t>
   </si>
   <si>
     <t xml:space="preserve">Q12</t>
@@ -596,7 +596,7 @@
     <t xml:space="preserve">256,278</t>
   </si>
   <si>
-    <t xml:space="preserve">53,946</t>
+    <t xml:space="preserve">53,866</t>
   </si>
   <si>
     <t xml:space="preserve">Q13</t>
@@ -605,7 +605,7 @@
     <t xml:space="preserve">199,218</t>
   </si>
   <si>
-    <t xml:space="preserve">24,371</t>
+    <t xml:space="preserve">24,177</t>
   </si>
   <si>
     <t xml:space="preserve">Q14</t>
@@ -614,7 +614,7 @@
     <t xml:space="preserve">124,173</t>
   </si>
   <si>
-    <t xml:space="preserve">32,016</t>
+    <t xml:space="preserve">32,329</t>
   </si>
   <si>
     <t xml:space="preserve">S01</t>
@@ -623,7 +623,7 @@
     <t xml:space="preserve">189,663</t>
   </si>
   <si>
-    <t xml:space="preserve">41,802</t>
+    <t xml:space="preserve">41,291</t>
   </si>
   <si>
     <t xml:space="preserve">S02</t>
@@ -632,16 +632,13 @@
     <t xml:space="preserve">140,795</t>
   </si>
   <si>
-    <t xml:space="preserve">19,496</t>
-  </si>
-  <si>
     <t xml:space="preserve">S03</t>
   </si>
   <si>
     <t xml:space="preserve">164,723</t>
   </si>
   <si>
-    <t xml:space="preserve">14,362</t>
+    <t xml:space="preserve">14,469</t>
   </si>
 </sst>
 </file>
@@ -1065,203 +1062,203 @@
         <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>7</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C17" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D17" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C20" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D20" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C21" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D21" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22">
@@ -1303,88 +1300,88 @@
         <v>90</v>
       </c>
       <c r="D24" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B25" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C25" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D25" t="s">
-        <v>68</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B26" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C26" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D26" t="s">
-        <v>97</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B27" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C27" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D27" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B28" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C28" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D28" t="s">
-        <v>64</v>
+        <v>105</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B29" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C29" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D29" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B30" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C30" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D30" t="s">
         <v>83</v>
@@ -1392,142 +1389,142 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B31" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C31" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D31" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B32" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C32" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D32" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B33" t="s">
+        <v>122</v>
+      </c>
+      <c r="C33" t="s">
+        <v>123</v>
+      </c>
+      <c r="D33" t="s">
         <v>120</v>
-      </c>
-      <c r="C33" t="s">
-        <v>121</v>
-      </c>
-      <c r="D33" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B34" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C34" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D34" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B35" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D35" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B36" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C36" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D36" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B37" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B38" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C38" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D38" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C39" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D39" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B40" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C40" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D40" t="s">
-        <v>146</v>
+        <v>105</v>
       </c>
     </row>
     <row r="41">
@@ -1541,7 +1538,7 @@
         <v>149</v>
       </c>
       <c r="D41" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="42">
@@ -1555,7 +1552,7 @@
         <v>152</v>
       </c>
       <c r="D42" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="43">
@@ -1569,7 +1566,7 @@
         <v>155</v>
       </c>
       <c r="D43" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="44">
@@ -1611,7 +1608,7 @@
         <v>166</v>
       </c>
       <c r="D46" t="s">
-        <v>87</v>
+        <v>159</v>
       </c>
     </row>
     <row r="47">
@@ -1625,7 +1622,7 @@
         <v>169</v>
       </c>
       <c r="D47" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="48">
@@ -1653,7 +1650,7 @@
         <v>176</v>
       </c>
       <c r="D49" t="s">
-        <v>57</v>
+        <v>173</v>
       </c>
     </row>
     <row r="50">
@@ -1695,7 +1692,7 @@
         <v>185</v>
       </c>
       <c r="D52" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
     </row>
     <row r="53">
@@ -1723,7 +1720,7 @@
         <v>191</v>
       </c>
       <c r="D54" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="55">
@@ -1737,7 +1734,7 @@
         <v>194</v>
       </c>
       <c r="D55" t="s">
-        <v>146</v>
+        <v>91</v>
       </c>
     </row>
     <row r="56">
@@ -1765,7 +1762,7 @@
         <v>200</v>
       </c>
       <c r="D57" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="58">
@@ -1790,7 +1787,7 @@
         <v>205</v>
       </c>
       <c r="C59" t="s">
-        <v>206</v>
+        <v>188</v>
       </c>
       <c r="D59" t="s">
         <v>159</v>
@@ -1798,16 +1795,16 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
+        <v>206</v>
+      </c>
+      <c r="B60" t="s">
         <v>207</v>
       </c>
-      <c r="B60" t="s">
+      <c r="C60" t="s">
         <v>208</v>
       </c>
-      <c r="C60" t="s">
-        <v>209</v>
-      </c>
       <c r="D60" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>